<commit_message>
Redo network scaling as three-tier risk model (High 112 / Medium 400 / Low 400)
- High tier: 112 profile-matched stops at the survey-calibrated case rate
- Medium: next 400 stops by AM-peak throughput at 50% rate (assumption)
- Low: following 400 stops at 25% rate (assumption)
- Network totals: 912 stops carrying 76% of peak arrivals, ~346k annual
  cases, ~2,880 bus-h delay @30s, dOTP -0.35 to -0.85 pp on peak trips
- STUDY.md sections 1 and 8 updated; tier_summary.csv replaces
  network_scaling.csv; per-stop tier in network_stop_scores.csv
- Excel model: new NetworkTiers sheet with adjustable rate multipliers
  (formulas independently verified)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016L5LdgJBiosDe7YPTsB2AS
</commit_message>
<xml_diff>
--- a/analysis/parking_otp_impact_model.xlsx
+++ b/analysis/parking_otp_impact_model.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BaseData22Jul" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NetworkTiers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000%"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -105,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,6 +145,10 @@
     <xf numFmtId="10" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1333,4 +1339,316 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Network-wide three-tier risk model (GTFS-based)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>High = 112 profile-matched stops; Medium/Low = next 400 / following 400 by AM-peak throughput. Rate multipliers are assumptions - adjust the blue cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GTFS AM-peak arrivals at the 27 surveyed stops</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="n">
+        <v>2084</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Calibrated case rate per AM-peak arrival</t>
+        </is>
+      </c>
+      <c r="B4" s="26">
+        <f>Assumptions!B5/B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Weekday bus trips with a peak-hour stop event</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n">
+        <v>9771</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Stops</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>AM-peak arrivals</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Rate multiplier</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Cases per AM peak</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Annual cases</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Delay hours @30s</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Extra late trips/yr @30s</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>Extra late trips/yr @60s</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>dOTP peak (pp) @30s</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>dOTP peak (pp) @60s</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>High (profile-matched)</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>112</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>12622</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="23">
+        <f>C8*$B$4*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="23">
+        <f>E8*(1+Assumptions!B8)*Assumptions!B10</f>
+        <v/>
+      </c>
+      <c r="G8" s="23">
+        <f>F8*Assumptions!B9/3600</f>
+        <v/>
+      </c>
+      <c r="H8" s="23">
+        <f>F8*Model!$B$16</f>
+        <v/>
+      </c>
+      <c r="I8" s="23">
+        <f>F8*Model!$B$17</f>
+        <v/>
+      </c>
+      <c r="J8" s="24">
+        <f>100*H8/($B$5*Assumptions!B10)</f>
+        <v/>
+      </c>
+      <c r="K8" s="24">
+        <f>100*I8/($B$5*Assumptions!B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Medium (next 400 by throughput)</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>18657</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="23">
+        <f>C9*$B$4*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="23">
+        <f>E9*(1+Assumptions!B8)*Assumptions!B10</f>
+        <v/>
+      </c>
+      <c r="G9" s="23">
+        <f>F9*Assumptions!B9/3600</f>
+        <v/>
+      </c>
+      <c r="H9" s="23">
+        <f>F9*Model!$B$16</f>
+        <v/>
+      </c>
+      <c r="I9" s="23">
+        <f>F9*Model!$B$17</f>
+        <v/>
+      </c>
+      <c r="J9" s="24">
+        <f>100*H9/($B$5*Assumptions!B10)</f>
+        <v/>
+      </c>
+      <c r="K9" s="24">
+        <f>100*I9/($B$5*Assumptions!B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Low (following 400)</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>8273</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E10" s="23">
+        <f>C10*$B$4*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="23">
+        <f>E10*(1+Assumptions!B8)*Assumptions!B10</f>
+        <v/>
+      </c>
+      <c r="G10" s="23">
+        <f>F10*Assumptions!B9/3600</f>
+        <v/>
+      </c>
+      <c r="H10" s="23">
+        <f>F10*Model!$B$16</f>
+        <v/>
+      </c>
+      <c r="I10" s="23">
+        <f>F10*Model!$B$17</f>
+        <v/>
+      </c>
+      <c r="J10" s="24">
+        <f>100*H10/($B$5*Assumptions!B10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="24">
+        <f>100*I10/($B$5*Assumptions!B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="27">
+        <f>SUM(B8:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="27">
+        <f>SUM(C8:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="27">
+        <f>SUM(E8:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="27">
+        <f>SUM(F8:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="27">
+        <f>SUM(G8:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="27">
+        <f>SUM(H8:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="27">
+        <f>SUM(I8:I10)</f>
+        <v/>
+      </c>
+      <c r="J11" s="28">
+        <f>SUM(J8:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="28">
+        <f>SUM(K8:K10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Cases = arrivals x calibrated rate x multiplier; annual = x (1+PM factor) x operating days. Flip probabilities referenced from Model sheet (22 Jul 2026 AVL). Source: analysis/network_scoring.py -&gt; tier_summary.csv</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add kerb monetization to model/study; rebuild deck on user's RTA-branded version
- roi_model.py: Option C kerb monetization - 2,000 permits at AED 1,200/yr
  + 1,000 ANPR-billed dwells/day at AED 5, ramp 40/80/100%, AED 2M platform
  capex + 0.5M/yr admin -> +10.2M NPV, payback yr 2, 4.2M/yr steady
- Excel model: new KerbMonetization sheet (recalculated, 130 formulas OK)
- STUDY.md: Option C section, monetization benchmarks (airport kerb fees,
  smart loading zones, Westminster coach bays, TNC zone surcharges),
  programme NPV ~+98M
- Deck rebuilt on the user's edited version as base: RTA logo throughout,
  new title design, exec summary tiles/band styling, 'Recommended' panel,
  ADCB Metro, Thank-you closer; adds monetization slide, kerb benchmark
  slide, and full-programme timeline (+119M cumulative, +98M NPV)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016L5LdgJBiosDe7YPTsB2AS
</commit_message>
<xml_diff>
--- a/analysis/parking_otp_impact_model.xlsx
+++ b/analysis/parking_otp_impact_model.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Model" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="NetworkTiers" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="ROI" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="KerbMonetization" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="131">
   <si>
     <t xml:space="preserve">Illegal Parking at Bus Stops - OTP Impact Model</t>
   </si>
@@ -357,6 +358,66 @@
   </si>
   <si>
     <t xml:space="preserve">Deterrence decay makes revenue decline by design - the permanent return is OTP recovery and safety. AED 500 federal fine scales revenue x2.5. Fine-revenue retention by RTA unconfirmed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kerb monetization - charging private operators for legal layby use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permits + ANPR-billed pay-per-use. Rides on the enforcement cameras (no extra field hardware). Blue = inputs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permitted vehicles (licensed operators)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit fee (AED/vehicle/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid dwells per day (network-wide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fee per dwell (AED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adoption ramp year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adoption ramp year 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adoption ramp year 3+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platform capex (AED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administration opex (AED/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady-state revenue (AED/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ramp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue (AED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opex (AED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net (AED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PV @ discount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5-yr NPV (AED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benchmarks: US airport kerb-access fees (USD 2.50-5/pick-up via geofence), smart loading zones (Pittsburgh, LA, Columbus - camera-billed per minute), Westminster paid coach bays. Source: analysis/roi_model.py</t>
   </si>
 </sst>
 </file>
@@ -515,7 +576,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -645,6 +706,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2249,4 +2318,286 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="29" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" s="29" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="29" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" s="30" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12" s="29" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="18" t="n">
+        <f aca="false">ROI!B10</f>
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" s="18" t="n">
+        <f aca="false">B4*B5+B6*B7*365</f>
+        <v>4225000</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="33" t="n">
+        <f aca="false">B8</f>
+        <v>0.4</v>
+      </c>
+      <c r="C18" s="23" t="n">
+        <f aca="false">$B$15*B18</f>
+        <v>1690000</v>
+      </c>
+      <c r="D18" s="23" t="n">
+        <f aca="false">$B$12</f>
+        <v>500000</v>
+      </c>
+      <c r="E18" s="23" t="n">
+        <f aca="false">C18-D18</f>
+        <v>1190000</v>
+      </c>
+      <c r="F18" s="23" t="n">
+        <f aca="false">E18/(1+$B$13)^A18</f>
+        <v>1112149.53271028</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="33" t="n">
+        <f aca="false">B9</f>
+        <v>0.8</v>
+      </c>
+      <c r="C19" s="23" t="n">
+        <f aca="false">$B$15*B19</f>
+        <v>3380000</v>
+      </c>
+      <c r="D19" s="23" t="n">
+        <f aca="false">$B$12</f>
+        <v>500000</v>
+      </c>
+      <c r="E19" s="23" t="n">
+        <f aca="false">C19-D19</f>
+        <v>2880000</v>
+      </c>
+      <c r="F19" s="23" t="n">
+        <f aca="false">E19/(1+$B$13)^A19</f>
+        <v>2515503.53742685</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="33" t="n">
+        <f aca="false">B10</f>
+        <v>1</v>
+      </c>
+      <c r="C20" s="23" t="n">
+        <f aca="false">$B$15*B20</f>
+        <v>4225000</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <f aca="false">$B$12</f>
+        <v>500000</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <f aca="false">C20-D20</f>
+        <v>3725000</v>
+      </c>
+      <c r="F20" s="23" t="n">
+        <f aca="false">E20/(1+$B$13)^A20</f>
+        <v>3040709.59141842</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="33" t="n">
+        <f aca="false">B10</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="23" t="n">
+        <f aca="false">$B$15*B21</f>
+        <v>4225000</v>
+      </c>
+      <c r="D21" s="23" t="n">
+        <f aca="false">$B$12</f>
+        <v>500000</v>
+      </c>
+      <c r="E21" s="23" t="n">
+        <f aca="false">C21-D21</f>
+        <v>3725000</v>
+      </c>
+      <c r="F21" s="23" t="n">
+        <f aca="false">E21/(1+$B$13)^A21</f>
+        <v>2841784.66487703</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="33" t="n">
+        <f aca="false">B10</f>
+        <v>1</v>
+      </c>
+      <c r="C22" s="23" t="n">
+        <f aca="false">$B$15*B22</f>
+        <v>4225000</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <f aca="false">$B$12</f>
+        <v>500000</v>
+      </c>
+      <c r="E22" s="23" t="n">
+        <f aca="false">C22-D22</f>
+        <v>3725000</v>
+      </c>
+      <c r="F22" s="23" t="n">
+        <f aca="false">E22/(1+$B$13)^A22</f>
+        <v>2655873.51857666</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="F23" s="34" t="n">
+        <f aca="false">SUM(F18:F22)-B11</f>
+        <v>10166020.8450092</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>